<commit_message>
Finalize Task 4 assessment report and evidence
</commit_message>
<xml_diff>
--- a/Money_Mitra_Network_Task4_Evidence_Workbook.xlsx
+++ b/Money_Mitra_Network_Task4_Evidence_Workbook.xlsx
@@ -1773,7 +1773,7 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Lab-Scans/task4-nmap.txt</t>
+          <t>Evidence/Lab-Scans/task4-nmap.txt</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1785,7 +1785,7 @@
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Lab-Scans/task4-targeted-checks.txt</t>
+          <t>Evidence/Lab-Scans/task4-targeted-checks.txt</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1797,7 +1797,7 @@
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Lab-Scans/task4-ftp-check.txt</t>
+          <t>Evidence/Lab-Scans/task4-ftp-check.txt</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1809,7 +1809,7 @@
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Lab-Scans/task4-http-headers.txt</t>
+          <t>Evidence/Lab-Scans/task4-http-headers.txt</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1821,7 +1821,7 @@
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>executable-http-details.tsv</t>
+          <t>Evidence/PCAP-Analysis/executable-http-details.tsv</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1833,7 +1833,7 @@
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>executable-verification.txt</t>
+          <t>Evidence/PCAP-Analysis/executable-verification.txt</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1845,7 +1845,7 @@
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>redirect-details.tsv</t>
+          <t>Evidence/PCAP-Analysis/redirect-details.tsv</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1857,7 +1857,7 @@
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>dns-error-responses.tsv</t>
+          <t>Evidence/PCAP-Analysis/dns-error-responses.tsv</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1869,7 +1869,7 @@
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Task4_Event_Timeline.txt</t>
+          <t>Evidence/Supporting-Files/Task4_Event_Timeline.txt</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1881,7 +1881,7 @@
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Task4_IOC_Table.csv</t>
+          <t>Evidence/Supporting-Files/Task4_IOC_Table.csv</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1893,7 +1893,7 @@
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Task4_Risk_Register.csv</t>
+          <t>Evidence/Supporting-Files/Task4_Risk_Register.csv</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1905,7 +1905,7 @@
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Task4_Detection_Rules.md</t>
+          <t>Evidence/Supporting-Files/Task4_Detection_Rules.md</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1917,7 +1917,7 @@
     <row r="14" ht="34" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Task4_Incident_Response_Plan.md</t>
+          <t>Evidence/Supporting-Files/Task4_Incident_Response_Plan.md</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>pcap-executable-download.png</t>
+          <t>Evidence/PCAP-Analysis/pcap-executable-download.png</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1941,7 +1941,7 @@
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>pcap-http-redirects.png</t>
+          <t>Evidence/PCAP-Analysis/pcap-http-redirects.png</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>pcap-long-connection.png</t>
+          <t>Evidence/PCAP-Analysis/pcap-long-connection.png</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1965,7 +1965,7 @@
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Lab-Scans/nmap-open-port.png</t>
+          <t>Evidence/Lab-Scans/nmap-open-port.png</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1977,7 +1977,7 @@
     <row r="19" ht="34" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Lab-Scans/nmap-remaning-ports.png</t>
+          <t>Evidence/Lab-Scans/nmap-remaning-ports.png</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1989,7 +1989,7 @@
     <row r="20" ht="34" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Lab-Scans/targeted-service-checks.png</t>
+          <t>Evidence/Lab-Scans/targeted-service-checks.png</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2001,7 +2001,7 @@
     <row r="21" ht="34" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Lab-Scans/ftp-anonymous-login.png</t>
+          <t>Evidence/Lab-Scans/ftp-anonymous-login.png</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2013,7 +2013,7 @@
     <row r="22" ht="34" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Lab-Scans/http-server-headers.png</t>
+          <t>Evidence/Lab-Scans/http-server-headers.png</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">

</xml_diff>